<commit_message>
Ajusta opções da planilha de atletas às listas do ScoutHub
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K3oSHiUMbMo7jeCvywkbmj
</commit_message>
<xml_diff>
--- a/atletas_importacao.xlsx
+++ b/atletas_importacao.xlsx
@@ -19,10 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -73,21 +72,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -590,7 +591,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="3" t="n">
+      <c r="F2" s="8" t="n">
         <v>41088</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -606,7 +607,7 @@
       <c r="I2" s="4" t="n">
         <v>1.91</v>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="J2" s="9" t="n">
         <v>86.2</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -666,7 +667,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="3" t="n">
+      <c r="F3" s="8" t="n">
         <v>39760</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -682,7 +683,7 @@
       <c r="I3" s="4" t="n">
         <v>1.83</v>
       </c>
-      <c r="J3" s="5" t="n">
+      <c r="J3" s="9" t="n">
         <v>77.2</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -746,7 +747,7 @@
           <t>Alemã</t>
         </is>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F4" s="8" t="n">
         <v>38652</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -762,7 +763,7 @@
       <c r="I4" s="4" t="n">
         <v>1.7</v>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="J4" s="9" t="n">
         <v>66.3</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -781,7 +782,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -822,7 +823,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="3" t="n">
+      <c r="F5" s="8" t="n">
         <v>35512</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -838,7 +839,7 @@
       <c r="I5" s="4" t="n">
         <v>1.76</v>
       </c>
-      <c r="J5" s="5" t="n">
+      <c r="J5" s="9" t="n">
         <v>74.3</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -898,7 +899,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="3" t="n">
+      <c r="F6" s="8" t="n">
         <v>40492</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -914,7 +915,7 @@
       <c r="I6" s="4" t="n">
         <v>1.84</v>
       </c>
-      <c r="J6" s="5" t="n">
+      <c r="J6" s="9" t="n">
         <v>84.2</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -974,7 +975,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="3" t="n">
+      <c r="F7" s="8" t="n">
         <v>40396</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -990,17 +991,17 @@
       <c r="I7" s="4" t="n">
         <v>1.81</v>
       </c>
-      <c r="J7" s="5" t="n">
+      <c r="J7" s="9" t="n">
         <v>79.2</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -1013,7 +1014,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1050,7 +1051,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="3" t="n">
+      <c r="F8" s="8" t="n">
         <v>39327</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1066,17 +1067,17 @@
       <c r="I8" s="4" t="n">
         <v>1.77</v>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="J8" s="9" t="n">
         <v>74.09999999999999</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1130,7 +1131,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="3" t="n">
+      <c r="F9" s="8" t="n">
         <v>33828</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1146,12 +1147,12 @@
       <c r="I9" s="4" t="n">
         <v>1.79</v>
       </c>
-      <c r="J9" s="5" t="n">
+      <c r="J9" s="9" t="n">
         <v>72.40000000000001</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1206,7 +1207,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="3" t="n">
+      <c r="F10" s="8" t="n">
         <v>40758</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1222,7 +1223,7 @@
       <c r="I10" s="4" t="n">
         <v>1.81</v>
       </c>
-      <c r="J10" s="5" t="n">
+      <c r="J10" s="9" t="n">
         <v>75.40000000000001</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1232,7 +1233,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1286,7 +1287,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="3" t="n">
+      <c r="F11" s="8" t="n">
         <v>39765</v>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1302,7 +1303,7 @@
       <c r="I11" s="4" t="n">
         <v>1.81</v>
       </c>
-      <c r="J11" s="5" t="n">
+      <c r="J11" s="9" t="n">
         <v>80.5</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1366,7 +1367,7 @@
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="3" t="n">
+      <c r="F12" s="8" t="n">
         <v>39047</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1382,17 +1383,17 @@
       <c r="I12" s="4" t="n">
         <v>1.83</v>
       </c>
-      <c r="J12" s="5" t="n">
+      <c r="J12" s="9" t="n">
         <v>81.5</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -1446,7 +1447,7 @@
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="3" t="n">
+      <c r="F13" s="8" t="n">
         <v>36235</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1462,12 +1463,12 @@
       <c r="I13" s="4" t="n">
         <v>1.75</v>
       </c>
-      <c r="J13" s="5" t="n">
+      <c r="J13" s="9" t="n">
         <v>68.3</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1485,7 +1486,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1526,7 +1527,7 @@
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="3" t="n">
+      <c r="F14" s="8" t="n">
         <v>40955</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1542,7 +1543,7 @@
       <c r="I14" s="4" t="n">
         <v>1.87</v>
       </c>
-      <c r="J14" s="5" t="n">
+      <c r="J14" s="9" t="n">
         <v>79.7</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1602,7 +1603,7 @@
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="3" t="n">
+      <c r="F15" s="8" t="n">
         <v>39951</v>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1618,7 +1619,7 @@
       <c r="I15" s="4" t="n">
         <v>1.74</v>
       </c>
-      <c r="J15" s="5" t="n">
+      <c r="J15" s="9" t="n">
         <v>68.59999999999999</v>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1628,7 +1629,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
@@ -1682,7 +1683,7 @@
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="3" t="n">
+      <c r="F16" s="8" t="n">
         <v>39633</v>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1698,7 +1699,7 @@
       <c r="I16" s="4" t="n">
         <v>1.7</v>
       </c>
-      <c r="J16" s="5" t="n">
+      <c r="J16" s="9" t="n">
         <v>62.6</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1717,7 +1718,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -1758,7 +1759,7 @@
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="3" t="n">
+      <c r="F17" s="8" t="n">
         <v>37235</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1774,7 +1775,7 @@
       <c r="I17" s="4" t="n">
         <v>1.82</v>
       </c>
-      <c r="J17" s="5" t="n">
+      <c r="J17" s="9" t="n">
         <v>79.59999999999999</v>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1830,7 +1831,7 @@
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="3" t="n">
+      <c r="F18" s="8" t="n">
         <v>40743</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1846,7 +1847,7 @@
       <c r="I18" s="4" t="n">
         <v>1.87</v>
       </c>
-      <c r="J18" s="5" t="n">
+      <c r="J18" s="9" t="n">
         <v>82.2</v>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1910,7 +1911,7 @@
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="3" t="n">
+      <c r="F19" s="8" t="n">
         <v>40461</v>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1926,7 +1927,7 @@
       <c r="I19" s="4" t="n">
         <v>1.76</v>
       </c>
-      <c r="J19" s="5" t="n">
+      <c r="J19" s="9" t="n">
         <v>73.40000000000001</v>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1936,7 +1937,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
@@ -1990,7 +1991,7 @@
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="3" t="n">
+      <c r="F20" s="8" t="n">
         <v>38951</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2006,17 +2007,17 @@
       <c r="I20" s="4" t="n">
         <v>1.82</v>
       </c>
-      <c r="J20" s="5" t="n">
+      <c r="J20" s="9" t="n">
         <v>78.8</v>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
@@ -2074,7 +2075,7 @@
           <t>Italiana</t>
         </is>
       </c>
-      <c r="F21" s="3" t="n">
+      <c r="F21" s="8" t="n">
         <v>37400</v>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -2090,17 +2091,17 @@
       <c r="I21" s="4" t="n">
         <v>1.71</v>
       </c>
-      <c r="J21" s="5" t="n">
+      <c r="J21" s="9" t="n">
         <v>68</v>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -2154,7 +2155,7 @@
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="3" t="n">
+      <c r="F22" s="8" t="n">
         <v>40823</v>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2170,17 +2171,17 @@
       <c r="I22" s="4" t="n">
         <v>1.75</v>
       </c>
-      <c r="J22" s="5" t="n">
+      <c r="J22" s="9" t="n">
         <v>69.3</v>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -2234,7 +2235,7 @@
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="3" t="n">
+      <c r="F23" s="8" t="n">
         <v>39977</v>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -2250,7 +2251,7 @@
       <c r="I23" s="4" t="n">
         <v>1.73</v>
       </c>
-      <c r="J23" s="5" t="n">
+      <c r="J23" s="9" t="n">
         <v>65.8</v>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2273,7 +2274,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
@@ -2314,7 +2315,7 @@
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="3" t="n">
+      <c r="F24" s="8" t="n">
         <v>39203</v>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2330,7 +2331,7 @@
       <c r="I24" s="4" t="n">
         <v>1.89</v>
       </c>
-      <c r="J24" s="5" t="n">
+      <c r="J24" s="9" t="n">
         <v>83.09999999999999</v>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2340,7 +2341,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -2353,7 +2354,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -2394,7 +2395,7 @@
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="3" t="n">
+      <c r="F25" s="8" t="n">
         <v>34513</v>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -2410,7 +2411,7 @@
       <c r="I25" s="4" t="n">
         <v>1.91</v>
       </c>
-      <c r="J25" s="5" t="n">
+      <c r="J25" s="9" t="n">
         <v>85.59999999999999</v>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -2420,7 +2421,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
@@ -2470,7 +2471,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="3" t="n">
+      <c r="F26" s="8" t="n">
         <v>38466</v>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -2486,7 +2487,7 @@
       <c r="I26" s="4" t="n">
         <v>1.88</v>
       </c>
-      <c r="J26" s="5" t="n">
+      <c r="J26" s="9" t="n">
         <v>84.8</v>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2546,7 +2547,7 @@
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="3" t="n">
+      <c r="F27" s="8" t="n">
         <v>40643</v>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -2562,7 +2563,7 @@
       <c r="I27" s="4" t="n">
         <v>1.93</v>
       </c>
-      <c r="J27" s="5" t="n">
+      <c r="J27" s="9" t="n">
         <v>88.90000000000001</v>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -2572,7 +2573,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
@@ -2585,7 +2586,7 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
@@ -2626,7 +2627,7 @@
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="3" t="n">
+      <c r="F28" s="8" t="n">
         <v>40323</v>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -2642,7 +2643,7 @@
       <c r="I28" s="4" t="n">
         <v>1.82</v>
       </c>
-      <c r="J28" s="5" t="n">
+      <c r="J28" s="9" t="n">
         <v>78.3</v>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -2698,7 +2699,7 @@
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
-      <c r="F29" s="3" t="n">
+      <c r="F29" s="8" t="n">
         <v>39831</v>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -2714,7 +2715,7 @@
       <c r="I29" s="4" t="n">
         <v>1.72</v>
       </c>
-      <c r="J29" s="5" t="n">
+      <c r="J29" s="9" t="n">
         <v>69.8</v>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -2724,7 +2725,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
@@ -2778,7 +2779,7 @@
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="3" t="n">
+      <c r="F30" s="8" t="n">
         <v>39323</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -2794,7 +2795,7 @@
       <c r="I30" s="4" t="n">
         <v>1.85</v>
       </c>
-      <c r="J30" s="5" t="n">
+      <c r="J30" s="9" t="n">
         <v>81.8</v>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -2858,7 +2859,7 @@
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
-      <c r="F31" s="3" t="n">
+      <c r="F31" s="8" t="n">
         <v>40678</v>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -2874,7 +2875,7 @@
       <c r="I31" s="4" t="n">
         <v>1.85</v>
       </c>
-      <c r="J31" s="5" t="n">
+      <c r="J31" s="9" t="n">
         <v>80.90000000000001</v>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -2884,7 +2885,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
@@ -2938,7 +2939,7 @@
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="3" t="n">
+      <c r="F32" s="8" t="n">
         <v>39168</v>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -2954,17 +2955,17 @@
       <c r="I32" s="4" t="n">
         <v>1.69</v>
       </c>
-      <c r="J32" s="5" t="n">
+      <c r="J32" s="9" t="n">
         <v>63</v>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
@@ -3014,7 +3015,7 @@
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr"/>
-      <c r="F33" s="3" t="n">
+      <c r="F33" s="8" t="n">
         <v>40034</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -3030,7 +3031,7 @@
       <c r="I33" s="4" t="n">
         <v>1.9</v>
       </c>
-      <c r="J33" s="5" t="n">
+      <c r="J33" s="9" t="n">
         <v>84</v>
       </c>
       <c r="K33" s="2" t="inlineStr">
@@ -3090,7 +3091,7 @@
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="3" t="n">
+      <c r="F34" s="8" t="n">
         <v>39927</v>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3106,17 +3107,17 @@
       <c r="I34" s="4" t="n">
         <v>1.69</v>
       </c>
-      <c r="J34" s="5" t="n">
+      <c r="J34" s="9" t="n">
         <v>62.5</v>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
@@ -3166,7 +3167,7 @@
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr"/>
-      <c r="F35" s="3" t="n">
+      <c r="F35" s="8" t="n">
         <v>40670</v>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -3182,7 +3183,7 @@
       <c r="I35" s="4" t="n">
         <v>1.95</v>
       </c>
-      <c r="J35" s="5" t="n">
+      <c r="J35" s="9" t="n">
         <v>93.7</v>
       </c>
       <c r="K35" s="2" t="inlineStr">
@@ -3238,7 +3239,7 @@
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="3" t="n">
+      <c r="F36" s="8" t="n">
         <v>40111</v>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -3254,7 +3255,7 @@
       <c r="I36" s="4" t="n">
         <v>1.75</v>
       </c>
-      <c r="J36" s="5" t="n">
+      <c r="J36" s="9" t="n">
         <v>70.59999999999999</v>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -3318,7 +3319,7 @@
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr"/>
-      <c r="F37" s="3" t="n">
+      <c r="F37" s="8" t="n">
         <v>34822</v>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -3334,12 +3335,12 @@
       <c r="I37" s="4" t="n">
         <v>1.73</v>
       </c>
-      <c r="J37" s="5" t="n">
+      <c r="J37" s="9" t="n">
         <v>67.5</v>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -3398,7 +3399,7 @@
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="3" t="n">
+      <c r="F38" s="8" t="n">
         <v>39967</v>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -3414,7 +3415,7 @@
       <c r="I38" s="4" t="n">
         <v>1.91</v>
       </c>
-      <c r="J38" s="5" t="n">
+      <c r="J38" s="9" t="n">
         <v>85.90000000000001</v>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -3424,7 +3425,7 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
@@ -3478,7 +3479,7 @@
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr"/>
-      <c r="F39" s="3" t="n">
+      <c r="F39" s="8" t="n">
         <v>38839</v>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -3494,12 +3495,12 @@
       <c r="I39" s="4" t="n">
         <v>1.71</v>
       </c>
-      <c r="J39" s="5" t="n">
+      <c r="J39" s="9" t="n">
         <v>68.3</v>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr"/>
@@ -3558,7 +3559,7 @@
           <t>Espanhola</t>
         </is>
       </c>
-      <c r="F40" s="3" t="n">
+      <c r="F40" s="8" t="n">
         <v>39847</v>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -3574,7 +3575,7 @@
       <c r="I40" s="4" t="n">
         <v>1.77</v>
       </c>
-      <c r="J40" s="5" t="n">
+      <c r="J40" s="9" t="n">
         <v>68.59999999999999</v>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -3584,7 +3585,7 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
@@ -3597,7 +3598,7 @@
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
@@ -3634,7 +3635,7 @@
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr"/>
-      <c r="F41" s="3" t="n">
+      <c r="F41" s="8" t="n">
         <v>40405</v>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -3650,7 +3651,7 @@
       <c r="I41" s="4" t="n">
         <v>1.95</v>
       </c>
-      <c r="J41" s="5" t="n">
+      <c r="J41" s="9" t="n">
         <v>94.09999999999999</v>
       </c>
       <c r="K41" s="2" t="inlineStr">
@@ -3706,7 +3707,7 @@
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="3" t="n">
+      <c r="F42" s="8" t="n">
         <v>40261</v>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -3722,12 +3723,12 @@
       <c r="I42" s="4" t="n">
         <v>1.79</v>
       </c>
-      <c r="J42" s="5" t="n">
+      <c r="J42" s="9" t="n">
         <v>77.59999999999999</v>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr"/>
@@ -3782,7 +3783,7 @@
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
-      <c r="F43" s="3" t="n">
+      <c r="F43" s="8" t="n">
         <v>41154</v>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -3798,12 +3799,12 @@
       <c r="I43" s="4" t="n">
         <v>1.77</v>
       </c>
-      <c r="J43" s="5" t="n">
+      <c r="J43" s="9" t="n">
         <v>73.40000000000001</v>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
@@ -3862,7 +3863,7 @@
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="3" t="n">
+      <c r="F44" s="8" t="n">
         <v>39468</v>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -3878,17 +3879,17 @@
       <c r="I44" s="4" t="n">
         <v>1.78</v>
       </c>
-      <c r="J44" s="5" t="n">
+      <c r="J44" s="9" t="n">
         <v>73.3</v>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M44" s="2" t="inlineStr">
@@ -3946,7 +3947,7 @@
           <t>Portuguesa</t>
         </is>
       </c>
-      <c r="F45" s="3" t="n">
+      <c r="F45" s="8" t="n">
         <v>38665</v>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -3962,7 +3963,7 @@
       <c r="I45" s="4" t="n">
         <v>1.71</v>
       </c>
-      <c r="J45" s="5" t="n">
+      <c r="J45" s="9" t="n">
         <v>64.5</v>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -4018,7 +4019,7 @@
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="3" t="n">
+      <c r="F46" s="8" t="n">
         <v>39128</v>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -4034,7 +4035,7 @@
       <c r="I46" s="4" t="n">
         <v>1.71</v>
       </c>
-      <c r="J46" s="5" t="n">
+      <c r="J46" s="9" t="n">
         <v>64.09999999999999</v>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -4053,7 +4054,7 @@
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr">
@@ -4098,7 +4099,7 @@
           <t>Alemã</t>
         </is>
       </c>
-      <c r="F47" s="3" t="n">
+      <c r="F47" s="8" t="n">
         <v>34353</v>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -4114,7 +4115,7 @@
       <c r="I47" s="4" t="n">
         <v>1.91</v>
       </c>
-      <c r="J47" s="5" t="n">
+      <c r="J47" s="9" t="n">
         <v>89.2</v>
       </c>
       <c r="K47" s="2" t="inlineStr">
@@ -4124,7 +4125,7 @@
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M47" s="2" t="inlineStr">
@@ -4178,7 +4179,7 @@
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr"/>
-      <c r="F48" s="3" t="n">
+      <c r="F48" s="8" t="n">
         <v>38569</v>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -4194,12 +4195,12 @@
       <c r="I48" s="4" t="n">
         <v>1.7</v>
       </c>
-      <c r="J48" s="5" t="n">
+      <c r="J48" s="9" t="n">
         <v>61.9</v>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
@@ -4217,7 +4218,7 @@
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P48" s="2" t="inlineStr">
@@ -4262,7 +4263,7 @@
           <t>Espanhola</t>
         </is>
       </c>
-      <c r="F49" s="3" t="n">
+      <c r="F49" s="8" t="n">
         <v>39866</v>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -4278,7 +4279,7 @@
       <c r="I49" s="4" t="n">
         <v>1.74</v>
       </c>
-      <c r="J49" s="5" t="n">
+      <c r="J49" s="9" t="n">
         <v>72.40000000000001</v>
       </c>
       <c r="K49" s="2" t="inlineStr">
@@ -4342,7 +4343,7 @@
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="3" t="n">
+      <c r="F50" s="8" t="n">
         <v>38392</v>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -4358,7 +4359,7 @@
       <c r="I50" s="4" t="n">
         <v>1.75</v>
       </c>
-      <c r="J50" s="5" t="n">
+      <c r="J50" s="9" t="n">
         <v>68.5</v>
       </c>
       <c r="K50" s="2" t="inlineStr">
@@ -4377,7 +4378,7 @@
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P50" s="2" t="inlineStr">
@@ -4418,7 +4419,7 @@
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr"/>
-      <c r="F51" s="3" t="n">
+      <c r="F51" s="8" t="n">
         <v>40189</v>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -4434,7 +4435,7 @@
       <c r="I51" s="4" t="n">
         <v>1.75</v>
       </c>
-      <c r="J51" s="5" t="n">
+      <c r="J51" s="9" t="n">
         <v>73.09999999999999</v>
       </c>
       <c r="K51" s="2" t="inlineStr">
@@ -4444,7 +4445,7 @@
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr">
@@ -4532,7 +4533,7 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Premissa: as opções de Posição Principal, Perna Dominante, Status Atual e Categoria não foram vistas no sistema; foram usados valores comuns do futebol. Ajuste se o sistema usar nomes diferentes.</t>
+          <t>Posição, Perna Dominante, Status e Categoria usam exatamente as opções do ScoutHub (ex.: Meio-campista, Meia Ofensivo, Ponta Direita/Esquerda, Livre).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajusta opções da planilha de atletas às listas do ScoutHub (#3)
Claude-Session: https://claude.ai/code/session_01K3oSHiUMbMo7jeCvywkbmj

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/atletas_importacao.xlsx
+++ b/atletas_importacao.xlsx
@@ -19,10 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -73,21 +72,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -590,7 +591,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="3" t="n">
+      <c r="F2" s="8" t="n">
         <v>41088</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -606,7 +607,7 @@
       <c r="I2" s="4" t="n">
         <v>1.91</v>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="J2" s="9" t="n">
         <v>86.2</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -666,7 +667,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="3" t="n">
+      <c r="F3" s="8" t="n">
         <v>39760</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -682,7 +683,7 @@
       <c r="I3" s="4" t="n">
         <v>1.83</v>
       </c>
-      <c r="J3" s="5" t="n">
+      <c r="J3" s="9" t="n">
         <v>77.2</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -746,7 +747,7 @@
           <t>Alemã</t>
         </is>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="F4" s="8" t="n">
         <v>38652</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -762,7 +763,7 @@
       <c r="I4" s="4" t="n">
         <v>1.7</v>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="J4" s="9" t="n">
         <v>66.3</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -781,7 +782,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -822,7 +823,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="3" t="n">
+      <c r="F5" s="8" t="n">
         <v>35512</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -838,7 +839,7 @@
       <c r="I5" s="4" t="n">
         <v>1.76</v>
       </c>
-      <c r="J5" s="5" t="n">
+      <c r="J5" s="9" t="n">
         <v>74.3</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -898,7 +899,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="3" t="n">
+      <c r="F6" s="8" t="n">
         <v>40492</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -914,7 +915,7 @@
       <c r="I6" s="4" t="n">
         <v>1.84</v>
       </c>
-      <c r="J6" s="5" t="n">
+      <c r="J6" s="9" t="n">
         <v>84.2</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -974,7 +975,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="3" t="n">
+      <c r="F7" s="8" t="n">
         <v>40396</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -990,17 +991,17 @@
       <c r="I7" s="4" t="n">
         <v>1.81</v>
       </c>
-      <c r="J7" s="5" t="n">
+      <c r="J7" s="9" t="n">
         <v>79.2</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -1013,7 +1014,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1050,7 +1051,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="3" t="n">
+      <c r="F8" s="8" t="n">
         <v>39327</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1066,17 +1067,17 @@
       <c r="I8" s="4" t="n">
         <v>1.77</v>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="J8" s="9" t="n">
         <v>74.09999999999999</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1130,7 +1131,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="3" t="n">
+      <c r="F9" s="8" t="n">
         <v>33828</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1146,12 +1147,12 @@
       <c r="I9" s="4" t="n">
         <v>1.79</v>
       </c>
-      <c r="J9" s="5" t="n">
+      <c r="J9" s="9" t="n">
         <v>72.40000000000001</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1206,7 +1207,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="3" t="n">
+      <c r="F10" s="8" t="n">
         <v>40758</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1222,7 +1223,7 @@
       <c r="I10" s="4" t="n">
         <v>1.81</v>
       </c>
-      <c r="J10" s="5" t="n">
+      <c r="J10" s="9" t="n">
         <v>75.40000000000001</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1232,7 +1233,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1286,7 +1287,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="3" t="n">
+      <c r="F11" s="8" t="n">
         <v>39765</v>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1302,7 +1303,7 @@
       <c r="I11" s="4" t="n">
         <v>1.81</v>
       </c>
-      <c r="J11" s="5" t="n">
+      <c r="J11" s="9" t="n">
         <v>80.5</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1366,7 +1367,7 @@
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="3" t="n">
+      <c r="F12" s="8" t="n">
         <v>39047</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1382,17 +1383,17 @@
       <c r="I12" s="4" t="n">
         <v>1.83</v>
       </c>
-      <c r="J12" s="5" t="n">
+      <c r="J12" s="9" t="n">
         <v>81.5</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -1446,7 +1447,7 @@
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="3" t="n">
+      <c r="F13" s="8" t="n">
         <v>36235</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1462,12 +1463,12 @@
       <c r="I13" s="4" t="n">
         <v>1.75</v>
       </c>
-      <c r="J13" s="5" t="n">
+      <c r="J13" s="9" t="n">
         <v>68.3</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1485,7 +1486,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1526,7 +1527,7 @@
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
-      <c r="F14" s="3" t="n">
+      <c r="F14" s="8" t="n">
         <v>40955</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1542,7 +1543,7 @@
       <c r="I14" s="4" t="n">
         <v>1.87</v>
       </c>
-      <c r="J14" s="5" t="n">
+      <c r="J14" s="9" t="n">
         <v>79.7</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1602,7 +1603,7 @@
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="3" t="n">
+      <c r="F15" s="8" t="n">
         <v>39951</v>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1618,7 +1619,7 @@
       <c r="I15" s="4" t="n">
         <v>1.74</v>
       </c>
-      <c r="J15" s="5" t="n">
+      <c r="J15" s="9" t="n">
         <v>68.59999999999999</v>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1628,7 +1629,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
@@ -1682,7 +1683,7 @@
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="3" t="n">
+      <c r="F16" s="8" t="n">
         <v>39633</v>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1698,7 +1699,7 @@
       <c r="I16" s="4" t="n">
         <v>1.7</v>
       </c>
-      <c r="J16" s="5" t="n">
+      <c r="J16" s="9" t="n">
         <v>62.6</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1717,7 +1718,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -1758,7 +1759,7 @@
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="3" t="n">
+      <c r="F17" s="8" t="n">
         <v>37235</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1774,7 +1775,7 @@
       <c r="I17" s="4" t="n">
         <v>1.82</v>
       </c>
-      <c r="J17" s="5" t="n">
+      <c r="J17" s="9" t="n">
         <v>79.59999999999999</v>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1830,7 +1831,7 @@
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="3" t="n">
+      <c r="F18" s="8" t="n">
         <v>40743</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1846,7 +1847,7 @@
       <c r="I18" s="4" t="n">
         <v>1.87</v>
       </c>
-      <c r="J18" s="5" t="n">
+      <c r="J18" s="9" t="n">
         <v>82.2</v>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1910,7 +1911,7 @@
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="3" t="n">
+      <c r="F19" s="8" t="n">
         <v>40461</v>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1926,7 +1927,7 @@
       <c r="I19" s="4" t="n">
         <v>1.76</v>
       </c>
-      <c r="J19" s="5" t="n">
+      <c r="J19" s="9" t="n">
         <v>73.40000000000001</v>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1936,7 +1937,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
@@ -1990,7 +1991,7 @@
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="3" t="n">
+      <c r="F20" s="8" t="n">
         <v>38951</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2006,17 +2007,17 @@
       <c r="I20" s="4" t="n">
         <v>1.82</v>
       </c>
-      <c r="J20" s="5" t="n">
+      <c r="J20" s="9" t="n">
         <v>78.8</v>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
@@ -2074,7 +2075,7 @@
           <t>Italiana</t>
         </is>
       </c>
-      <c r="F21" s="3" t="n">
+      <c r="F21" s="8" t="n">
         <v>37400</v>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -2090,17 +2091,17 @@
       <c r="I21" s="4" t="n">
         <v>1.71</v>
       </c>
-      <c r="J21" s="5" t="n">
+      <c r="J21" s="9" t="n">
         <v>68</v>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -2154,7 +2155,7 @@
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="3" t="n">
+      <c r="F22" s="8" t="n">
         <v>40823</v>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2170,17 +2171,17 @@
       <c r="I22" s="4" t="n">
         <v>1.75</v>
       </c>
-      <c r="J22" s="5" t="n">
+      <c r="J22" s="9" t="n">
         <v>69.3</v>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -2234,7 +2235,7 @@
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="3" t="n">
+      <c r="F23" s="8" t="n">
         <v>39977</v>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -2250,7 +2251,7 @@
       <c r="I23" s="4" t="n">
         <v>1.73</v>
       </c>
-      <c r="J23" s="5" t="n">
+      <c r="J23" s="9" t="n">
         <v>65.8</v>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2273,7 +2274,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
@@ -2314,7 +2315,7 @@
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="3" t="n">
+      <c r="F24" s="8" t="n">
         <v>39203</v>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2330,7 +2331,7 @@
       <c r="I24" s="4" t="n">
         <v>1.89</v>
       </c>
-      <c r="J24" s="5" t="n">
+      <c r="J24" s="9" t="n">
         <v>83.09999999999999</v>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2340,7 +2341,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -2353,7 +2354,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -2394,7 +2395,7 @@
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="3" t="n">
+      <c r="F25" s="8" t="n">
         <v>34513</v>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -2410,7 +2411,7 @@
       <c r="I25" s="4" t="n">
         <v>1.91</v>
       </c>
-      <c r="J25" s="5" t="n">
+      <c r="J25" s="9" t="n">
         <v>85.59999999999999</v>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -2420,7 +2421,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
@@ -2470,7 +2471,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="3" t="n">
+      <c r="F26" s="8" t="n">
         <v>38466</v>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -2486,7 +2487,7 @@
       <c r="I26" s="4" t="n">
         <v>1.88</v>
       </c>
-      <c r="J26" s="5" t="n">
+      <c r="J26" s="9" t="n">
         <v>84.8</v>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2546,7 +2547,7 @@
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="3" t="n">
+      <c r="F27" s="8" t="n">
         <v>40643</v>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -2562,7 +2563,7 @@
       <c r="I27" s="4" t="n">
         <v>1.93</v>
       </c>
-      <c r="J27" s="5" t="n">
+      <c r="J27" s="9" t="n">
         <v>88.90000000000001</v>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -2572,7 +2573,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
@@ -2585,7 +2586,7 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
@@ -2626,7 +2627,7 @@
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="3" t="n">
+      <c r="F28" s="8" t="n">
         <v>40323</v>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -2642,7 +2643,7 @@
       <c r="I28" s="4" t="n">
         <v>1.82</v>
       </c>
-      <c r="J28" s="5" t="n">
+      <c r="J28" s="9" t="n">
         <v>78.3</v>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -2698,7 +2699,7 @@
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr"/>
-      <c r="F29" s="3" t="n">
+      <c r="F29" s="8" t="n">
         <v>39831</v>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -2714,7 +2715,7 @@
       <c r="I29" s="4" t="n">
         <v>1.72</v>
       </c>
-      <c r="J29" s="5" t="n">
+      <c r="J29" s="9" t="n">
         <v>69.8</v>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -2724,7 +2725,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
@@ -2778,7 +2779,7 @@
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="3" t="n">
+      <c r="F30" s="8" t="n">
         <v>39323</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -2794,7 +2795,7 @@
       <c r="I30" s="4" t="n">
         <v>1.85</v>
       </c>
-      <c r="J30" s="5" t="n">
+      <c r="J30" s="9" t="n">
         <v>81.8</v>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -2858,7 +2859,7 @@
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr"/>
-      <c r="F31" s="3" t="n">
+      <c r="F31" s="8" t="n">
         <v>40678</v>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -2874,7 +2875,7 @@
       <c r="I31" s="4" t="n">
         <v>1.85</v>
       </c>
-      <c r="J31" s="5" t="n">
+      <c r="J31" s="9" t="n">
         <v>80.90000000000001</v>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -2884,7 +2885,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
@@ -2938,7 +2939,7 @@
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="3" t="n">
+      <c r="F32" s="8" t="n">
         <v>39168</v>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -2954,17 +2955,17 @@
       <c r="I32" s="4" t="n">
         <v>1.69</v>
       </c>
-      <c r="J32" s="5" t="n">
+      <c r="J32" s="9" t="n">
         <v>63</v>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
@@ -3014,7 +3015,7 @@
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr"/>
-      <c r="F33" s="3" t="n">
+      <c r="F33" s="8" t="n">
         <v>40034</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -3030,7 +3031,7 @@
       <c r="I33" s="4" t="n">
         <v>1.9</v>
       </c>
-      <c r="J33" s="5" t="n">
+      <c r="J33" s="9" t="n">
         <v>84</v>
       </c>
       <c r="K33" s="2" t="inlineStr">
@@ -3090,7 +3091,7 @@
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="3" t="n">
+      <c r="F34" s="8" t="n">
         <v>39927</v>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -3106,17 +3107,17 @@
       <c r="I34" s="4" t="n">
         <v>1.69</v>
       </c>
-      <c r="J34" s="5" t="n">
+      <c r="J34" s="9" t="n">
         <v>62.5</v>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
@@ -3166,7 +3167,7 @@
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr"/>
-      <c r="F35" s="3" t="n">
+      <c r="F35" s="8" t="n">
         <v>40670</v>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -3182,7 +3183,7 @@
       <c r="I35" s="4" t="n">
         <v>1.95</v>
       </c>
-      <c r="J35" s="5" t="n">
+      <c r="J35" s="9" t="n">
         <v>93.7</v>
       </c>
       <c r="K35" s="2" t="inlineStr">
@@ -3238,7 +3239,7 @@
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="3" t="n">
+      <c r="F36" s="8" t="n">
         <v>40111</v>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -3254,7 +3255,7 @@
       <c r="I36" s="4" t="n">
         <v>1.75</v>
       </c>
-      <c r="J36" s="5" t="n">
+      <c r="J36" s="9" t="n">
         <v>70.59999999999999</v>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -3318,7 +3319,7 @@
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr"/>
-      <c r="F37" s="3" t="n">
+      <c r="F37" s="8" t="n">
         <v>34822</v>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -3334,12 +3335,12 @@
       <c r="I37" s="4" t="n">
         <v>1.73</v>
       </c>
-      <c r="J37" s="5" t="n">
+      <c r="J37" s="9" t="n">
         <v>67.5</v>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -3398,7 +3399,7 @@
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="3" t="n">
+      <c r="F38" s="8" t="n">
         <v>39967</v>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -3414,7 +3415,7 @@
       <c r="I38" s="4" t="n">
         <v>1.91</v>
       </c>
-      <c r="J38" s="5" t="n">
+      <c r="J38" s="9" t="n">
         <v>85.90000000000001</v>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -3424,7 +3425,7 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M38" s="2" t="inlineStr">
@@ -3478,7 +3479,7 @@
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr"/>
-      <c r="F39" s="3" t="n">
+      <c r="F39" s="8" t="n">
         <v>38839</v>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -3494,12 +3495,12 @@
       <c r="I39" s="4" t="n">
         <v>1.71</v>
       </c>
-      <c r="J39" s="5" t="n">
+      <c r="J39" s="9" t="n">
         <v>68.3</v>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr"/>
@@ -3558,7 +3559,7 @@
           <t>Espanhola</t>
         </is>
       </c>
-      <c r="F40" s="3" t="n">
+      <c r="F40" s="8" t="n">
         <v>39847</v>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -3574,7 +3575,7 @@
       <c r="I40" s="4" t="n">
         <v>1.77</v>
       </c>
-      <c r="J40" s="5" t="n">
+      <c r="J40" s="9" t="n">
         <v>68.59999999999999</v>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -3584,7 +3585,7 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
@@ -3597,7 +3598,7 @@
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
@@ -3634,7 +3635,7 @@
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr"/>
-      <c r="F41" s="3" t="n">
+      <c r="F41" s="8" t="n">
         <v>40405</v>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -3650,7 +3651,7 @@
       <c r="I41" s="4" t="n">
         <v>1.95</v>
       </c>
-      <c r="J41" s="5" t="n">
+      <c r="J41" s="9" t="n">
         <v>94.09999999999999</v>
       </c>
       <c r="K41" s="2" t="inlineStr">
@@ -3706,7 +3707,7 @@
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="3" t="n">
+      <c r="F42" s="8" t="n">
         <v>40261</v>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -3722,12 +3723,12 @@
       <c r="I42" s="4" t="n">
         <v>1.79</v>
       </c>
-      <c r="J42" s="5" t="n">
+      <c r="J42" s="9" t="n">
         <v>77.59999999999999</v>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr"/>
@@ -3782,7 +3783,7 @@
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr"/>
-      <c r="F43" s="3" t="n">
+      <c r="F43" s="8" t="n">
         <v>41154</v>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -3798,12 +3799,12 @@
       <c r="I43" s="4" t="n">
         <v>1.77</v>
       </c>
-      <c r="J43" s="5" t="n">
+      <c r="J43" s="9" t="n">
         <v>73.40000000000001</v>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
@@ -3862,7 +3863,7 @@
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="3" t="n">
+      <c r="F44" s="8" t="n">
         <v>39468</v>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -3878,17 +3879,17 @@
       <c r="I44" s="4" t="n">
         <v>1.78</v>
       </c>
-      <c r="J44" s="5" t="n">
+      <c r="J44" s="9" t="n">
         <v>73.3</v>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Meia Atacante</t>
+          <t>Meia Ofensivo</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M44" s="2" t="inlineStr">
@@ -3946,7 +3947,7 @@
           <t>Portuguesa</t>
         </is>
       </c>
-      <c r="F45" s="3" t="n">
+      <c r="F45" s="8" t="n">
         <v>38665</v>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -3962,7 +3963,7 @@
       <c r="I45" s="4" t="n">
         <v>1.71</v>
       </c>
-      <c r="J45" s="5" t="n">
+      <c r="J45" s="9" t="n">
         <v>64.5</v>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -4018,7 +4019,7 @@
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="3" t="n">
+      <c r="F46" s="8" t="n">
         <v>39128</v>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -4034,7 +4035,7 @@
       <c r="I46" s="4" t="n">
         <v>1.71</v>
       </c>
-      <c r="J46" s="5" t="n">
+      <c r="J46" s="9" t="n">
         <v>64.09999999999999</v>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -4053,7 +4054,7 @@
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr">
@@ -4098,7 +4099,7 @@
           <t>Alemã</t>
         </is>
       </c>
-      <c r="F47" s="3" t="n">
+      <c r="F47" s="8" t="n">
         <v>34353</v>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -4114,7 +4115,7 @@
       <c r="I47" s="4" t="n">
         <v>1.91</v>
       </c>
-      <c r="J47" s="5" t="n">
+      <c r="J47" s="9" t="n">
         <v>89.2</v>
       </c>
       <c r="K47" s="2" t="inlineStr">
@@ -4124,7 +4125,7 @@
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M47" s="2" t="inlineStr">
@@ -4178,7 +4179,7 @@
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr"/>
-      <c r="F48" s="3" t="n">
+      <c r="F48" s="8" t="n">
         <v>38569</v>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -4194,12 +4195,12 @@
       <c r="I48" s="4" t="n">
         <v>1.7</v>
       </c>
-      <c r="J48" s="5" t="n">
+      <c r="J48" s="9" t="n">
         <v>61.9</v>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Meia</t>
+          <t>Meio-campista</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
@@ -4217,7 +4218,7 @@
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P48" s="2" t="inlineStr">
@@ -4262,7 +4263,7 @@
           <t>Espanhola</t>
         </is>
       </c>
-      <c r="F49" s="3" t="n">
+      <c r="F49" s="8" t="n">
         <v>39866</v>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -4278,7 +4279,7 @@
       <c r="I49" s="4" t="n">
         <v>1.74</v>
       </c>
-      <c r="J49" s="5" t="n">
+      <c r="J49" s="9" t="n">
         <v>72.40000000000001</v>
       </c>
       <c r="K49" s="2" t="inlineStr">
@@ -4342,7 +4343,7 @@
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="3" t="n">
+      <c r="F50" s="8" t="n">
         <v>38392</v>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -4358,7 +4359,7 @@
       <c r="I50" s="4" t="n">
         <v>1.75</v>
       </c>
-      <c r="J50" s="5" t="n">
+      <c r="J50" s="9" t="n">
         <v>68.5</v>
       </c>
       <c r="K50" s="2" t="inlineStr">
@@ -4377,7 +4378,7 @@
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>Livre no mercado</t>
+          <t>Livre</t>
         </is>
       </c>
       <c r="P50" s="2" t="inlineStr">
@@ -4418,7 +4419,7 @@
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr"/>
-      <c r="F51" s="3" t="n">
+      <c r="F51" s="8" t="n">
         <v>40189</v>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -4434,7 +4435,7 @@
       <c r="I51" s="4" t="n">
         <v>1.75</v>
       </c>
-      <c r="J51" s="5" t="n">
+      <c r="J51" s="9" t="n">
         <v>73.09999999999999</v>
       </c>
       <c r="K51" s="2" t="inlineStr">
@@ -4444,7 +4445,7 @@
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>Ponta</t>
+          <t>Ponta Direita</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr">
@@ -4532,7 +4533,7 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Premissa: as opções de Posição Principal, Perna Dominante, Status Atual e Categoria não foram vistas no sistema; foram usados valores comuns do futebol. Ajuste se o sistema usar nomes diferentes.</t>
+          <t>Posição, Perna Dominante, Status e Categoria usam exatamente as opções do ScoutHub (ex.: Meio-campista, Meia Ofensivo, Ponta Direita/Esquerda, Livre).</t>
         </is>
       </c>
     </row>

</xml_diff>